<commit_message>
Keep auto filter criteria, dxf references, chart style and zero-width columns
- Auto filters with filter columns or sort state are exported as {"ref", "xml"}.
- Differential formats referenced by tables and auto filters are exported per
  sheet (dxfs) and renumbered on import.
- Chart style and rounded corners are restored.
- Columns with width 0 keep it.
- Example 03 table column names match their header cells.
- New test_xml_paths checks that no XML element or attribute of an example
  vanishes in a round-trip.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UZs6wsi5TT3GKqgC7bYeY
</commit_message>
<xml_diff>
--- a/examples/01-basic-data.xlsx
+++ b/examples/01-basic-data.xlsx
@@ -95,6 +95,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -467,6 +476,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col hidden="1" width="8" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col hidden="1" min="9" max="9" width="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -671,7 +681,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>Консультація 06</t>
@@ -865,7 +875,7 @@
         </is>
       </c>
     </row>
-    <row r="13" outlineLevel="1">
+    <row r="13" hidden="1" outlineLevel="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>Консультація 12</t>
@@ -1059,7 +1069,7 @@
         </is>
       </c>
     </row>
-    <row r="19" outlineLevel="1">
+    <row r="19" hidden="1" outlineLevel="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>Консультація 18</t>
@@ -1447,7 +1457,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="1">
       <c r="A31" t="inlineStr">
         <is>
           <t>Консультація 30</t>
@@ -1641,7 +1651,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>Консультація 36</t>
@@ -1802,7 +1812,20 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H41"/>
+  <autoFilter ref="A1:H41">
+    <filterColumn colId="1" hiddenButton="0" showButton="1">
+      <filters>
+        <filter val="Hardware"/>
+        <filter val="Services"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="6" hiddenButton="0" showButton="1">
+      <colorFilter dxfId="0"/>
+    </filterColumn>
+    <sortState ref="A2:H41">
+      <sortCondition descending="1" ref="D2:D41"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>